<commit_message>
Update Документ “perechen-smsp” +1
</commit_message>
<xml_diff>
--- a/public/uploads/perechen-zakupok-smsp.xlsx
+++ b/public/uploads/perechen-zakupok-smsp.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\moscollector.local\docs\ООЗ\ЗАКУПКИ 2026\ПЕРЕЧЕНЬ ЗАКУПОК У СМСП\Корректировка 4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\moscollector.local\docs\ООЗ\ЗАКУПКИ 2026\ПЕРЕЧЕНЬ ЗАКУПОК У СМСП\Корректировка 5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA9620E1-932E-4FFA-A297-C890D603DAA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B80C5173-FCE0-49BD-AB84-A0288316BAA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="750" yWindow="885" windowWidth="25350" windowHeight="13995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Лист1!$A$8:$C$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Лист1!$A$1:$C$286</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Лист1!$A$1:$C$291</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="553">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="561">
   <si>
     <t>ОКПД 2</t>
   </si>
@@ -1714,13 +1714,37 @@
     <t>Пленки прочие пластмассовые пористые</t>
   </si>
   <si>
-    <t xml:space="preserve">Первый заместитель генерального директора              </t>
-  </si>
-  <si>
-    <t xml:space="preserve">                                                                      М.В. Епифанцев</t>
-  </si>
-  <si>
-    <t>к приказу от 14.05.2026 № 186</t>
+    <t xml:space="preserve">31.02.10.120 </t>
+  </si>
+  <si>
+    <t>Шкафы кухонные</t>
+  </si>
+  <si>
+    <t>31.02.10.190</t>
+  </si>
+  <si>
+    <t>Мебель кухонная прочая</t>
+  </si>
+  <si>
+    <t>31.09.12.131</t>
+  </si>
+  <si>
+    <t>Столы обеденные деревянные для столовой и гостиной</t>
+  </si>
+  <si>
+    <t>81.22.12.000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Услуги по чистке и уборке специализированные </t>
+  </si>
+  <si>
+    <t>61.20.50.110</t>
+  </si>
+  <si>
+    <t>Услуги связи для целей эфирного вещания</t>
+  </si>
+  <si>
+    <t>к приказу от 16.06.2026 № 237</t>
   </si>
 </sst>
 </file>
@@ -1855,7 +1879,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1963,6 +1987,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2315,7 +2343,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J284"/>
+  <dimension ref="A1:J289"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="12" customWidth="1"/>
@@ -2332,7 +2360,7 @@
     </row>
     <row r="2" spans="1:4" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C2" s="39" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2342,21 +2370,21 @@
       <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:4" ht="3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="43" t="s">
         <v>335</v>
       </c>
-      <c r="B5" s="41"/>
-      <c r="C5" s="41"/>
+      <c r="B5" s="43"/>
+      <c r="C5" s="43"/>
     </row>
     <row r="6" spans="1:4" ht="2.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="41"/>
-      <c r="B6" s="41"/>
-      <c r="C6" s="41"/>
+      <c r="A6" s="43"/>
+      <c r="B6" s="43"/>
+      <c r="C6" s="43"/>
     </row>
     <row r="7" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="42"/>
-      <c r="B7" s="42"/>
-      <c r="C7" s="42"/>
+      <c r="A7" s="44"/>
+      <c r="B7" s="44"/>
+      <c r="C7" s="44"/>
     </row>
     <row r="8" spans="1:4" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
@@ -4710,7 +4738,7 @@
     </row>
     <row r="204" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="5">
-        <f t="shared" ref="A204:A267" si="3">A203+1</f>
+        <f t="shared" ref="A204:A213" si="3">A203+1</f>
         <v>196</v>
       </c>
       <c r="B204" s="5" t="s">
@@ -4828,842 +4856,824 @@
         <v>538</v>
       </c>
     </row>
-    <row r="214" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A214" s="5">
-        <f t="shared" si="3"/>
         <v>206</v>
       </c>
       <c r="B214" s="5" t="s">
+        <v>550</v>
+      </c>
+      <c r="C214" s="42" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A215" s="5">
+        <v>207</v>
+      </c>
+      <c r="B215" s="5" t="s">
+        <v>552</v>
+      </c>
+      <c r="C215" s="7" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A216" s="5">
+        <v>208</v>
+      </c>
+      <c r="B216" s="5" t="s">
         <v>419</v>
       </c>
-      <c r="C214" s="7" t="s">
+      <c r="C216" s="7" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="215" spans="1:3" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A215" s="5">
-        <f t="shared" si="3"/>
-        <v>207</v>
-      </c>
-      <c r="B215" s="24" t="s">
+    <row r="217" spans="1:3" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A217" s="5">
+        <v>209</v>
+      </c>
+      <c r="B217" s="24" t="s">
         <v>455</v>
       </c>
-      <c r="C215" s="9" t="s">
+      <c r="C217" s="9" t="s">
         <v>456</v>
       </c>
     </row>
-    <row r="216" spans="1:3" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A216" s="5">
-        <f t="shared" si="3"/>
-        <v>208</v>
-      </c>
-      <c r="B216" s="24" t="s">
+    <row r="218" spans="1:3" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A218" s="5">
+        <v>210</v>
+      </c>
+      <c r="B218" s="24" t="s">
         <v>523</v>
       </c>
-      <c r="C216" s="9" t="s">
+      <c r="C218" s="9" t="s">
         <v>524</v>
       </c>
     </row>
-    <row r="217" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A217" s="5">
-        <f t="shared" si="3"/>
-        <v>209</v>
-      </c>
-      <c r="B217" s="5" t="s">
+    <row r="219" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A219" s="5">
+        <v>211</v>
+      </c>
+      <c r="B219" s="5" t="s">
+        <v>554</v>
+      </c>
+      <c r="C219" s="7" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A220" s="5">
+        <v>212</v>
+      </c>
+      <c r="B220" s="5" t="s">
         <v>421</v>
       </c>
-      <c r="C217" s="7" t="s">
+      <c r="C220" s="7" t="s">
         <v>422</v>
       </c>
     </row>
-    <row r="218" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A218" s="5">
-        <f t="shared" si="3"/>
-        <v>210</v>
-      </c>
-      <c r="B218" s="5" t="s">
+    <row r="221" spans="1:3" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A221" s="5">
+        <v>213</v>
+      </c>
+      <c r="B221" s="5" t="s">
         <v>525</v>
       </c>
-      <c r="C218" s="7" t="s">
+      <c r="C221" s="7" t="s">
         <v>526</v>
       </c>
     </row>
-    <row r="219" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A219" s="5">
-        <f t="shared" si="3"/>
-        <v>211</v>
-      </c>
-      <c r="B219" s="5" t="s">
+    <row r="222" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A222" s="5">
+        <v>214</v>
+      </c>
+      <c r="B222" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="C219" s="7" t="s">
+      <c r="C222" s="7" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A220" s="5">
-        <f t="shared" si="3"/>
-        <v>212</v>
-      </c>
-      <c r="B220" s="5" t="s">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A223" s="5">
+        <v>215</v>
+      </c>
+      <c r="B223" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="C220" s="7" t="s">
+      <c r="C223" s="7" t="s">
         <v>334</v>
-      </c>
-    </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A221" s="5">
-        <f t="shared" si="3"/>
-        <v>213</v>
-      </c>
-      <c r="B221" s="6" t="s">
-        <v>318</v>
-      </c>
-      <c r="C221" s="7" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A222" s="5">
-        <f t="shared" si="3"/>
-        <v>214</v>
-      </c>
-      <c r="B222" s="6" t="s">
-        <v>320</v>
-      </c>
-      <c r="C222" s="7" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="223" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A223" s="5">
-        <f t="shared" si="3"/>
-        <v>215</v>
-      </c>
-      <c r="B223" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="C223" s="9" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" s="5">
-        <f t="shared" si="3"/>
         <v>216</v>
       </c>
       <c r="B224" s="6" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="C224" s="7" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="225" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" s="5">
-        <f t="shared" si="3"/>
         <v>217</v>
       </c>
       <c r="B225" s="6" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="C225" s="7" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A226" s="5">
-        <f t="shared" si="3"/>
         <v>218</v>
       </c>
-      <c r="B226" s="6" t="s">
-        <v>326</v>
-      </c>
-      <c r="C226" s="7" t="s">
-        <v>327</v>
+      <c r="B226" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C226" s="9" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227" s="5">
-        <f t="shared" si="3"/>
         <v>219</v>
       </c>
       <c r="B227" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="C227" s="7" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A228" s="5">
+        <v>220</v>
+      </c>
+      <c r="B228" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="C228" s="7" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A229" s="5">
+        <v>221</v>
+      </c>
+      <c r="B229" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="C229" s="7" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A230" s="5">
+        <v>222</v>
+      </c>
+      <c r="B230" s="6" t="s">
         <v>328</v>
       </c>
-      <c r="C227" s="7" t="s">
+      <c r="C230" s="7" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="228" spans="1:3" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A228" s="5">
-        <f t="shared" si="3"/>
-        <v>220</v>
-      </c>
-      <c r="B228" s="5" t="s">
+    <row r="231" spans="1:3" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A231" s="5">
+        <v>223</v>
+      </c>
+      <c r="B231" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="C228" s="7" t="s">
+      <c r="C231" s="7" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="229" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A229" s="5">
-        <f t="shared" si="3"/>
-        <v>221</v>
-      </c>
-      <c r="B229" s="5" t="s">
+    <row r="232" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A232" s="5">
+        <v>224</v>
+      </c>
+      <c r="B232" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C229" s="7" t="s">
+      <c r="C232" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="230" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A230" s="5">
-        <f t="shared" si="3"/>
-        <v>222</v>
-      </c>
-      <c r="B230" s="5" t="s">
+    <row r="233" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A233" s="5">
+        <v>225</v>
+      </c>
+      <c r="B233" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="C230" s="7" t="s">
+      <c r="C233" s="7" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="231" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A231" s="5">
-        <f t="shared" si="3"/>
-        <v>223</v>
-      </c>
-      <c r="B231" s="5" t="s">
+    <row r="234" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A234" s="5">
+        <v>226</v>
+      </c>
+      <c r="B234" s="5" t="s">
         <v>387</v>
       </c>
-      <c r="C231" s="7" t="s">
+      <c r="C234" s="7" t="s">
         <v>388</v>
-      </c>
-    </row>
-    <row r="232" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A232" s="5">
-        <f t="shared" si="3"/>
-        <v>224</v>
-      </c>
-      <c r="B232" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="C232" s="7" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="233" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A233" s="5">
-        <f t="shared" si="3"/>
-        <v>225</v>
-      </c>
-      <c r="B233" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="C233" s="7" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="234" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A234" s="5">
-        <f t="shared" si="3"/>
-        <v>226</v>
-      </c>
-      <c r="B234" s="8" t="s">
-        <v>382</v>
-      </c>
-      <c r="C234" s="7" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="235" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A235" s="5">
-        <f t="shared" si="3"/>
         <v>227</v>
       </c>
       <c r="B235" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C235" s="7" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="236" spans="1:3" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A236" s="5">
+        <v>228</v>
+      </c>
+      <c r="B236" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="C236" s="7" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A237" s="5">
+        <v>229</v>
+      </c>
+      <c r="B237" s="8" t="s">
+        <v>382</v>
+      </c>
+      <c r="C237" s="7" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A238" s="5">
+        <v>230</v>
+      </c>
+      <c r="B238" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="C235" s="7" t="s">
+      <c r="C238" s="7" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="236" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A236" s="5">
-        <f t="shared" si="3"/>
-        <v>228</v>
-      </c>
-      <c r="B236" s="5" t="s">
+    <row r="239" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A239" s="5">
+        <v>231</v>
+      </c>
+      <c r="B239" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="C236" s="7" t="s">
+      <c r="C239" s="7" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="237" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A237" s="5">
-        <f t="shared" si="3"/>
-        <v>229</v>
-      </c>
-      <c r="B237" s="8" t="s">
+    <row r="240" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A240" s="5">
+        <v>232</v>
+      </c>
+      <c r="B240" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="C237" s="7" t="s">
+      <c r="C240" s="7" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="238" spans="1:3" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A238" s="5">
-        <f t="shared" si="3"/>
-        <v>230</v>
-      </c>
-      <c r="B238" s="8" t="s">
+    <row r="241" spans="1:3" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A241" s="5">
+        <v>233</v>
+      </c>
+      <c r="B241" s="8" t="s">
         <v>384</v>
       </c>
-      <c r="C238" s="7" t="s">
+      <c r="C241" s="7" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="239" spans="1:3" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A239" s="5">
-        <f t="shared" si="3"/>
-        <v>231</v>
-      </c>
-      <c r="B239" s="8" t="s">
+    <row r="242" spans="1:3" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A242" s="5">
+        <v>234</v>
+      </c>
+      <c r="B242" s="8" t="s">
         <v>360</v>
       </c>
-      <c r="C239" s="7" t="s">
+      <c r="C242" s="7" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="240" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A240" s="5">
-        <f t="shared" si="3"/>
-        <v>232</v>
-      </c>
-      <c r="B240" s="8" t="s">
+    <row r="243" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A243" s="5">
+        <v>235</v>
+      </c>
+      <c r="B243" s="8" t="s">
         <v>409</v>
       </c>
-      <c r="C240" s="7" t="s">
+      <c r="C243" s="7" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="241" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A241" s="5">
-        <f t="shared" si="3"/>
-        <v>233</v>
-      </c>
-      <c r="B241" s="8" t="s">
+    <row r="244" spans="1:3" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A244" s="5">
+        <v>236</v>
+      </c>
+      <c r="B244" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C241" s="7" t="s">
+      <c r="C244" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="242" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A242" s="5">
-        <f t="shared" si="3"/>
-        <v>234</v>
-      </c>
-      <c r="B242" s="8" t="s">
+    <row r="245" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A245" s="5">
+        <v>237</v>
+      </c>
+      <c r="B245" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C242" s="7" t="s">
+      <c r="C245" s="7" t="s">
         <v>149</v>
-      </c>
-    </row>
-    <row r="243" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A243" s="5">
-        <f t="shared" si="3"/>
-        <v>235</v>
-      </c>
-      <c r="B243" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="C243" s="7" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A244" s="5">
-        <f t="shared" si="3"/>
-        <v>236</v>
-      </c>
-      <c r="B244" s="5" t="s">
-        <v>358</v>
-      </c>
-      <c r="C244" s="7" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="245" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A245" s="5">
-        <f t="shared" si="3"/>
-        <v>237</v>
-      </c>
-      <c r="B245" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="C245" s="7" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="246" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A246" s="5">
-        <f t="shared" si="3"/>
         <v>238</v>
       </c>
       <c r="B246" s="5" t="s">
-        <v>246</v>
+        <v>153</v>
       </c>
       <c r="C246" s="7" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="247" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" s="5">
-        <f t="shared" si="3"/>
         <v>239</v>
       </c>
-      <c r="B247" s="8" t="s">
-        <v>10</v>
+      <c r="B247" s="5" t="s">
+        <v>358</v>
       </c>
       <c r="C247" s="7" t="s">
-        <v>11</v>
+        <v>359</v>
       </c>
     </row>
     <row r="248" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A248" s="5">
-        <f t="shared" si="3"/>
         <v>240</v>
       </c>
-      <c r="B248" s="8" t="s">
+      <c r="B248" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="C248" s="7" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A249" s="5">
+        <v>241</v>
+      </c>
+      <c r="B249" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="C249" s="7" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="250" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A250" s="5">
+        <v>242</v>
+      </c>
+      <c r="B250" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C250" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="251" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A251" s="5">
+        <v>243</v>
+      </c>
+      <c r="B251" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C248" s="7" t="s">
+      <c r="C251" s="7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A249" s="5">
-        <f t="shared" si="3"/>
-        <v>241</v>
-      </c>
-      <c r="B249" s="8" t="s">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A252" s="5">
+        <v>244</v>
+      </c>
+      <c r="B252" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="C249" s="7" t="s">
+      <c r="C252" s="7" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A250" s="5">
-        <f t="shared" si="3"/>
-        <v>242</v>
-      </c>
-      <c r="B250" s="8" t="s">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A253" s="5">
+        <v>245</v>
+      </c>
+      <c r="B253" s="8" t="s">
         <v>386</v>
       </c>
-      <c r="C250" s="7" t="s">
+      <c r="C253" s="7" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A251" s="5">
-        <f t="shared" si="3"/>
-        <v>243</v>
-      </c>
-      <c r="B251" s="8" t="s">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A254" s="5">
+        <v>246</v>
+      </c>
+      <c r="B254" s="8" t="s">
         <v>236</v>
       </c>
-      <c r="C251" s="7" t="s">
+      <c r="C254" s="7" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="252" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A252" s="5">
-        <f t="shared" si="3"/>
-        <v>244</v>
-      </c>
-      <c r="B252" s="8" t="s">
+    <row r="255" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A255" s="5">
+        <v>247</v>
+      </c>
+      <c r="B255" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="C252" s="9" t="s">
+      <c r="C255" s="9" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="253" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A253" s="5">
-        <f t="shared" si="3"/>
-        <v>245</v>
-      </c>
-      <c r="B253" s="8" t="s">
+    <row r="256" spans="1:3" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A256" s="5">
+        <v>248</v>
+      </c>
+      <c r="B256" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="C253" s="9" t="s">
+      <c r="C256" s="9" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="254" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A254" s="5">
-        <f t="shared" si="3"/>
-        <v>246</v>
-      </c>
-      <c r="B254" s="8" t="s">
+    <row r="257" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A257" s="5">
+        <v>249</v>
+      </c>
+      <c r="B257" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="C254" s="9" t="s">
+      <c r="C257" s="9" t="s">
         <v>134</v>
-      </c>
-    </row>
-    <row r="255" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A255" s="5">
-        <f t="shared" si="3"/>
-        <v>247</v>
-      </c>
-      <c r="B255" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="C255" s="9" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="256" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A256" s="5">
-        <f t="shared" si="3"/>
-        <v>248</v>
-      </c>
-      <c r="B256" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="C256" s="9" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A257" s="5">
-        <f t="shared" si="3"/>
-        <v>249</v>
-      </c>
-      <c r="B257" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="C257" s="9" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="258" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A258" s="5">
-        <f t="shared" si="3"/>
         <v>250</v>
       </c>
       <c r="B258" s="8" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="C258" s="9" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="259" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A259" s="5">
-        <f t="shared" si="3"/>
         <v>251</v>
       </c>
-      <c r="B259" s="8" t="s">
-        <v>143</v>
+      <c r="B259" s="5" t="s">
+        <v>137</v>
       </c>
       <c r="C259" s="9" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="260" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" s="5">
-        <f t="shared" si="3"/>
         <v>252</v>
       </c>
       <c r="B260" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="C260" s="7" t="s">
-        <v>4</v>
+        <v>139</v>
+      </c>
+      <c r="C260" s="9" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="261" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A261" s="5">
-        <f t="shared" si="3"/>
         <v>253</v>
       </c>
       <c r="B261" s="8" t="s">
-        <v>221</v>
-      </c>
-      <c r="C261" s="7" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.3">
+        <v>141</v>
+      </c>
+      <c r="C261" s="9" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" s="5">
-        <f t="shared" si="3"/>
         <v>254</v>
       </c>
-      <c r="B262" s="31" t="s">
-        <v>527</v>
-      </c>
-      <c r="C262" s="7" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B262" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="C262" s="9" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A263" s="5">
-        <f t="shared" si="3"/>
         <v>255</v>
       </c>
       <c r="B263" s="8" t="s">
-        <v>354</v>
+        <v>2</v>
       </c>
       <c r="C263" s="7" t="s">
-        <v>355</v>
+        <v>4</v>
       </c>
     </row>
     <row r="264" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A264" s="5">
-        <f t="shared" si="3"/>
         <v>256</v>
       </c>
       <c r="B264" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="C264" s="7" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A265" s="5">
+        <v>257</v>
+      </c>
+      <c r="B265" s="31" t="s">
+        <v>527</v>
+      </c>
+      <c r="C265" s="7" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A266" s="5">
+        <v>258</v>
+      </c>
+      <c r="B266" s="8" t="s">
+        <v>354</v>
+      </c>
+      <c r="C266" s="7" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A267" s="5">
+        <v>259</v>
+      </c>
+      <c r="B267" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="C264" s="7" t="s">
+      <c r="C267" s="7" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="265" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A265" s="5">
-        <f t="shared" si="3"/>
-        <v>257</v>
-      </c>
-      <c r="B265" s="8" t="s">
+    <row r="268" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A268" s="5">
+        <v>260</v>
+      </c>
+      <c r="B268" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C265" s="7" t="s">
+      <c r="C268" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="266" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A266" s="5">
-        <f t="shared" si="3"/>
-        <v>258</v>
-      </c>
-      <c r="B266" s="8" t="s">
+    <row r="269" spans="1:3" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A269" s="24">
+        <v>261</v>
+      </c>
+      <c r="B269" s="41" t="s">
+        <v>558</v>
+      </c>
+      <c r="C269" s="9" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="270" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A270" s="5">
+        <v>262</v>
+      </c>
+      <c r="B270" s="8" t="s">
         <v>356</v>
       </c>
-      <c r="C266" s="7" t="s">
+      <c r="C270" s="7" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="267" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A267" s="5">
-        <f t="shared" si="3"/>
-        <v>259</v>
-      </c>
-      <c r="B267" s="8" t="s">
+    <row r="271" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A271" s="5">
+        <v>263</v>
+      </c>
+      <c r="B271" s="8" t="s">
         <v>453</v>
       </c>
-      <c r="C267" s="7" t="s">
+      <c r="C271" s="7" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="268" spans="1:3" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A268" s="5">
-        <f t="shared" ref="A268:A281" si="4">A267+1</f>
-        <v>260</v>
-      </c>
-      <c r="B268" s="8" t="s">
+    <row r="272" spans="1:3" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A272" s="5">
+        <v>264</v>
+      </c>
+      <c r="B272" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C268" s="7" t="s">
+      <c r="C272" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="269" spans="1:3" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A269" s="5">
-        <f t="shared" si="4"/>
-        <v>261</v>
-      </c>
-      <c r="B269" s="29" t="s">
+    <row r="273" spans="1:10" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A273" s="5">
+        <v>265</v>
+      </c>
+      <c r="B273" s="29" t="s">
         <v>489</v>
       </c>
-      <c r="C269" s="28" t="s">
+      <c r="C273" s="28" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="270" spans="1:3" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A270" s="5">
-        <f t="shared" si="4"/>
-        <v>262</v>
-      </c>
-      <c r="B270" s="8" t="s">
+    <row r="274" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A274" s="5">
+        <v>266</v>
+      </c>
+      <c r="B274" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C270" s="7" t="s">
+      <c r="C274" s="7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="271" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A271" s="5">
-        <f t="shared" si="4"/>
-        <v>263</v>
-      </c>
-      <c r="B271" s="5" t="s">
+    <row r="275" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A275" s="5">
+        <v>267</v>
+      </c>
+      <c r="B275" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="C271" s="7" t="s">
+      <c r="C275" s="7" t="s">
         <v>151</v>
-      </c>
-    </row>
-    <row r="272" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A272" s="5">
-        <f t="shared" si="4"/>
-        <v>264</v>
-      </c>
-      <c r="B272" s="6" t="s">
-        <v>330</v>
-      </c>
-      <c r="C272" s="7" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="273" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A273" s="5">
-        <f t="shared" si="4"/>
-        <v>265</v>
-      </c>
-      <c r="B273" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="C273" s="7" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="274" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A274" s="5">
-        <f t="shared" si="4"/>
-        <v>266</v>
-      </c>
-      <c r="B274" s="5" t="s">
-        <v>423</v>
-      </c>
-      <c r="C274" s="7" t="s">
-        <v>424</v>
-      </c>
-      <c r="J274" s="21"/>
-    </row>
-    <row r="275" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A275" s="5">
-        <f t="shared" si="4"/>
-        <v>267</v>
-      </c>
-      <c r="B275" s="5" t="s">
-        <v>239</v>
-      </c>
-      <c r="C275" s="7" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="276" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A276" s="5">
-        <f t="shared" si="4"/>
         <v>268</v>
       </c>
-      <c r="B276" s="5" t="s">
-        <v>200</v>
+      <c r="B276" s="6" t="s">
+        <v>330</v>
       </c>
       <c r="C276" s="7" t="s">
-        <v>201</v>
+        <v>331</v>
       </c>
     </row>
     <row r="277" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A277" s="5">
-        <f t="shared" si="4"/>
         <v>269</v>
       </c>
       <c r="B277" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="C277" s="7" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="278" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A278" s="5">
+        <v>270</v>
+      </c>
+      <c r="B278" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="C278" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="J278" s="21"/>
+    </row>
+    <row r="279" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A279" s="5">
+        <v>271</v>
+      </c>
+      <c r="B279" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="C279" s="7" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="280" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A280" s="5">
+        <v>272</v>
+      </c>
+      <c r="B280" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="C280" s="7" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="281" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A281" s="5">
+        <v>273</v>
+      </c>
+      <c r="B281" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C277" s="7" t="s">
+      <c r="C281" s="7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="278" spans="1:10" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A278" s="5">
-        <f t="shared" si="4"/>
-        <v>270</v>
-      </c>
-      <c r="B278" s="5" t="s">
+    <row r="282" spans="1:10" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A282" s="5">
+        <v>274</v>
+      </c>
+      <c r="B282" s="5" t="s">
         <v>437</v>
       </c>
-      <c r="C278" s="22" t="s">
+      <c r="C282" s="22" t="s">
         <v>438</v>
       </c>
     </row>
-    <row r="279" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A279" s="5">
-        <f t="shared" si="4"/>
-        <v>271</v>
-      </c>
-      <c r="B279" s="5" t="s">
+    <row r="283" spans="1:10" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A283" s="5">
+        <v>275</v>
+      </c>
+      <c r="B283" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="C279" s="7" t="s">
+      <c r="C283" s="7" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="280" spans="1:10" s="25" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A280" s="5">
-        <f t="shared" si="4"/>
-        <v>272</v>
-      </c>
-      <c r="B280" s="5" t="s">
+    <row r="284" spans="1:10" s="25" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A284" s="5">
+        <v>276</v>
+      </c>
+      <c r="B284" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="C284" s="23" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="285" spans="1:10" s="25" customFormat="1" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A285" s="5">
+        <v>277</v>
+      </c>
+      <c r="B285" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C280" s="23" t="s">
+      <c r="C285" s="23" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="281" spans="1:10" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A281" s="5">
-        <f t="shared" si="4"/>
-        <v>273</v>
-      </c>
-      <c r="B281" s="5" t="s">
+    <row r="286" spans="1:10" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A286" s="5">
+        <v>278</v>
+      </c>
+      <c r="B286" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="C281" s="7" t="s">
+      <c r="C286" s="7" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="282" spans="1:10" ht="15" x14ac:dyDescent="0.25">
-      <c r="A282" s="1"/>
-      <c r="B282" s="1"/>
-      <c r="C282" s="1"/>
-    </row>
-    <row r="284" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A284" s="12" t="s">
-        <v>550</v>
-      </c>
-      <c r="C284" s="40" t="s">
-        <v>551</v>
-      </c>
-      <c r="D284" s="36"/>
-      <c r="E284" s="37"/>
-      <c r="F284" s="37"/>
-      <c r="G284" s="38"/>
-      <c r="H284" s="12"/>
-      <c r="I284" s="12"/>
-      <c r="J284" s="12"/>
+    <row r="287" spans="1:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="A287" s="1"/>
+      <c r="B287" s="1"/>
+      <c r="C287" s="1"/>
+    </row>
+    <row r="289" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C289" s="40"/>
+      <c r="D289" s="36"/>
+      <c r="E289" s="37"/>
+      <c r="F289" s="37"/>
+      <c r="G289" s="38"/>
+      <c r="H289" s="12"/>
+      <c r="I289" s="12"/>
+      <c r="J289" s="12"/>
     </row>
   </sheetData>
   <autoFilter ref="A8:C8" xr:uid="{00000000-0009-0000-0000-000000000000}">
@@ -5676,10 +5686,6 @@
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="66" fitToHeight="0" orientation="portrait" r:id="rId1"/>
-  <rowBreaks count="2" manualBreakCount="2">
-    <brk id="36" max="2" man="1"/>
-    <brk id="234" max="2" man="1"/>
-  </rowBreaks>
 </worksheet>
 </file>
 

</xml_diff>